<commit_message>
feat(commissions-notifications): agregar comisiones de super admin en importador Excel y notificaciones por correo a fcb@creditonegocios.com.mx
</commit_message>
<xml_diff>
--- a/Plantilla_Productos_por_Financiera.xlsx
+++ b/Plantilla_Productos_por_Financiera.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AI3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -468,33 +468,42 @@
         <v>tiempo_respuesta</v>
       </c>
       <c r="W1" t="str">
+        <v>comision_apertura_superadmin</v>
+      </c>
+      <c r="X1" t="str">
+        <v>comision_sobretasa_superadmin</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>comision_renovacion_superadmin</v>
+      </c>
+      <c r="Z1" t="str">
         <v>comision_apertura_broker</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AA1" t="str">
         <v>comision_sobretasa_broker</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AB1" t="str">
         <v>comision_renovacion_broker</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AC1" t="str">
         <v>comision_apertura_master</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>comision_sobretasa_master</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>comision_renovacion_master</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AF1" t="str">
         <v>contacto</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AG1" t="str">
         <v>email_contacto</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AH1" t="str">
         <v>telefono_contacto</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AI1" t="str">
         <v>observaciones</v>
       </c>
     </row>
@@ -566,33 +575,42 @@
         <v>24-48 horas</v>
       </c>
       <c r="W2">
+        <v>3</v>
+      </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
+      <c r="Y2">
+        <v>0.5</v>
+      </c>
+      <c r="Z2">
         <v>1.5</v>
       </c>
-      <c r="X2">
+      <c r="AA2">
         <v>0.5</v>
       </c>
-      <c r="Y2">
+      <c r="AB2">
         <v>0.3</v>
       </c>
-      <c r="Z2">
+      <c r="AC2">
         <v>0.5</v>
       </c>
-      <c r="AA2">
+      <c r="AD2">
         <v>0.2</v>
       </c>
-      <c r="AB2">
+      <c r="AE2">
         <v>0.1</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AF2" t="str">
         <v>Equipo Comercial</v>
       </c>
-      <c r="AD2" t="str">
+      <c r="AG2" t="str">
         <v>contacto@financiera.com</v>
       </c>
-      <c r="AE2" t="str">
+      <c r="AH2" t="str">
         <v>5512345678</v>
       </c>
-      <c r="AF2" t="str">
+      <c r="AI2" t="str">
         <v>Una fila equivale a un producto por financiera para un perfil</v>
       </c>
     </row>
@@ -664,39 +682,48 @@
         <v>48-72 horas</v>
       </c>
       <c r="W3">
+        <v>2.5</v>
+      </c>
+      <c r="X3">
+        <v>0.8</v>
+      </c>
+      <c r="Y3">
+        <v>0.4</v>
+      </c>
+      <c r="Z3">
         <v>1.2</v>
       </c>
-      <c r="X3">
+      <c r="AA3">
         <v>0.4</v>
       </c>
-      <c r="Y3">
+      <c r="AB3">
         <v>0.2</v>
       </c>
-      <c r="Z3">
+      <c r="AC3">
         <v>0.4</v>
       </c>
-      <c r="AA3">
+      <c r="AD3">
         <v>0.2</v>
       </c>
-      <c r="AB3">
+      <c r="AE3">
         <v>0.1</v>
       </c>
-      <c r="AC3" t="str">
+      <c r="AF3" t="str">
         <v>Equipo PYME</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AG3" t="str">
         <v>pyme@financiera.com</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AH3" t="str">
         <v>5587654321</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AI3" t="str">
         <v>Mismo producto, perfil distinto -&gt; fila distinta</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AI3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>